<commit_message>
Update analysis pipeline outputs
</commit_message>
<xml_diff>
--- a/data/processed/sea_ice_extent_12_month_forecast.xlsx
+++ b/data/processed/sea_ice_extent_12_month_forecast.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>mean</t>
   </si>
@@ -26,6 +26,9 @@
   </si>
   <si>
     <t>mean_ci_upper</t>
+  </si>
+  <si>
+    <t>date</t>
   </si>
 </sst>
 </file>
@@ -393,6 +396,9 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
+      <c r="A1" s="1" t="s">
+        <v>4</v>
+      </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>

</xml_diff>